<commit_message>
Adding known future capacity retirements
</commit_message>
<xml_diff>
--- a/VerveStacks_EST/SuppXLS/Scen_known_elk_retirements.xlsx
+++ b/VerveStacks_EST/SuppXLS/Scen_known_elk_retirements.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\PycharmProjects\ee-times\VerveStacks_EST\SuppXLS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CDE8B799-81CB-4BAD-BC07-98A228EA5155}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7B77B03A-5FCB-4475-8B06-19E921A2712C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-10470" yWindow="10890" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="retired_capacity" sheetId="1" r:id="rId1"/>
@@ -27,25 +27,25 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
   <si>
-    <t>~TFM_INS</t>
-  </si>
-  <si>
     <t>Attribute</t>
   </si>
   <si>
     <t>Process</t>
   </si>
   <si>
-    <t>Year</t>
-  </si>
-  <si>
-    <t>Value</t>
-  </si>
-  <si>
-    <t>NCAP_BND</t>
-  </si>
-  <si>
     <t>ep_coal_cfb_balti</t>
+  </si>
+  <si>
+    <t>~TFM_INS-TS</t>
+  </si>
+  <si>
+    <t>limtype</t>
+  </si>
+  <si>
+    <t>up</t>
+  </si>
+  <si>
+    <t>CAP_BND</t>
   </si>
 </sst>
 </file>
@@ -368,22 +368,23 @@
   <cols>
     <col min="1" max="1" width="27.7109375" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="16.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>1</v>
       </c>
-      <c r="B3" t="s">
-        <v>2</v>
+      <c r="B3">
+        <v>2030</v>
       </c>
       <c r="C3" t="s">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="D3" t="s">
         <v>4</v>
@@ -391,16 +392,16 @@
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
+        <v>2</v>
+      </c>
+      <c r="B4">
+        <v>0</v>
+      </c>
+      <c r="C4" t="s">
+        <v>6</v>
+      </c>
+      <c r="D4" t="s">
         <v>5</v>
-      </c>
-      <c r="B4" t="s">
-        <v>6</v>
-      </c>
-      <c r="C4">
-        <v>2030</v>
-      </c>
-      <c r="D4">
-        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>